<commit_message>
chore: alinear reportes y comandos por servicio
</commit_message>
<xml_diff>
--- a/PLAN_DE_PRUEBAS_RENDIMIENTO_SI058_2026-05.xlsx
+++ b/PLAN_DE_PRUEBAS_RENDIMIENTO_SI058_2026-05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="92">
   <si>
     <t>N°</t>
   </si>
@@ -52,7 +52,7 @@
     <t>Smoke</t>
   </si>
   <si>
-    <t>npm run perf:carnet:smoke</t>
+    <t>npm run smoke:carnet</t>
   </si>
   <si>
     <t>1 IP / 1 VU / 4 iteraciones / CSV Carnet.</t>
@@ -73,7 +73,7 @@
     <t>Audit (Multi-IP)</t>
   </si>
   <si>
-    <t>npm run perf:audit</t>
+    <t>npm run perf:carnet:audit</t>
   </si>
   <si>
     <t>10 IPs (.48-.57) / Usuarios 2-11 / CSV Carnet.</t>
@@ -91,7 +91,7 @@
     <t>Baseline / Load</t>
   </si>
   <si>
-    <t>npm run perf:cp02</t>
+    <t>npm run perf:carnet:cp02</t>
   </si>
   <si>
     <t>11 IPs / 11 VUs / 10 iteraciones por VU.</t>
@@ -109,7 +109,7 @@
     <t>Stress (Ramping)</t>
   </si>
   <si>
-    <t>npm run perf:stress</t>
+    <t>npm run perf:carnet:stress</t>
   </si>
   <si>
     <t>10 IPs / Escalera de carga hasta 50 VUs configurable.</t>
@@ -127,7 +127,7 @@
     <t>WAF Limit</t>
   </si>
   <si>
-    <t>npm run perf:cp01</t>
+    <t>npm run perf:carnet:cp01</t>
   </si>
   <si>
     <t>1 IP / Ramping arrival rate configurable (default 5 -&gt; 20 RPS).</t>
@@ -145,7 +145,7 @@
     <t>Breakpoint / Stress Extreme</t>
   </si>
   <si>
-    <t>npm run perf:cp03</t>
+    <t>npm run perf:carnet:cp03</t>
   </si>
   <si>
     <t>500 VUs default / 10 IPs / sin think time / escalado agresivo.</t>
@@ -163,7 +163,7 @@
     <t>Collapse / Breakpoint Rápido</t>
   </si>
   <si>
-    <t>npm run perf:collapse</t>
+    <t>npm run perf:carnet:collapse</t>
   </si>
   <si>
     <t>Rampa rápida hasta 800 VUs default / solo endpoint Carné.</t>
@@ -181,7 +181,7 @@
     <t>Spike</t>
   </si>
   <si>
-    <t>npm run perf:spike</t>
+    <t>npm run perf:carnet:spike</t>
   </si>
   <si>
     <t>Rampa súbita configurable hasta 50 VUs default.</t>
@@ -199,7 +199,7 @@
     <t>Soak / Endurance</t>
   </si>
   <si>
-    <t>npm run perf:soak</t>
+    <t>npm run perf:carnet:soak</t>
   </si>
   <si>
     <t>10 VUs default durante 30 minutos configurable.</t>
@@ -214,7 +214,7 @@
     <t>Grados</t>
   </si>
   <si>
-    <t>npm run perf:grados:smoke</t>
+    <t>npm run smoke:grados</t>
   </si>
   <si>
     <t>1 IP / 1 VU / 4 iteraciones / CSV Grados.</t>
@@ -287,117 +287,6 @@
   </si>
   <si>
     <t>npm run perf:grados:soak</t>
-  </si>
-  <si>
-    <t>CP-MIX-01</t>
-  </si>
-  <si>
-    <t>Carné + Grados</t>
-  </si>
-  <si>
-    <t>Carga Mixta Realista</t>
-  </si>
-  <si>
-    <t>Mixed Load</t>
-  </si>
-  <si>
-    <t>npm run perf:all:load</t>
-  </si>
-  <si>
-    <t>Tráfico mixto configurable; default 70% Carné / 30% Grados.</t>
-  </si>
-  <si>
-    <t>Validar comportamiento del sistema con proporción realista de uso y SLO global.</t>
-  </si>
-  <si>
-    <t>CP-MIX-02</t>
-  </si>
-  <si>
-    <t>Stress Mixto</t>
-  </si>
-  <si>
-    <t>Mixed Stress</t>
-  </si>
-  <si>
-    <t>npm run perf:all:stress</t>
-  </si>
-  <si>
-    <t>Tráfico mixto 70/30 default con rampa hasta 50 VUs configurable.</t>
-  </si>
-  <si>
-    <t>Identificar degradación cruzada entre endpoints y módulo que se degrada primero.</t>
-  </si>
-  <si>
-    <t>CP-MIX-03</t>
-  </si>
-  <si>
-    <t>Spike Mixto</t>
-  </si>
-  <si>
-    <t>Mixed Spike</t>
-  </si>
-  <si>
-    <t>npm run perf:all:spike</t>
-  </si>
-  <si>
-    <t>Pico repentino con tráfico mixto 70/30 default.</t>
-  </si>
-  <si>
-    <t>Validar resiliencia del sistema completo ante pico súbito y recuperación.</t>
-  </si>
-  <si>
-    <t>CP-MIX-04</t>
-  </si>
-  <si>
-    <t>Soak Mixto</t>
-  </si>
-  <si>
-    <t>Mixed Soak</t>
-  </si>
-  <si>
-    <t>npm run perf:all:soak</t>
-  </si>
-  <si>
-    <t>Carga mixta sostenida durante 30 minutos default.</t>
-  </si>
-  <si>
-    <t>Detectar degradación gradual, contención de recursos compartidos y fatiga del backend.</t>
-  </si>
-  <si>
-    <t>CP-MIX-05</t>
-  </si>
-  <si>
-    <t>Saturación Sistémica</t>
-  </si>
-  <si>
-    <t>Mixed Breakpoint</t>
-  </si>
-  <si>
-    <t>npm run perf:all:cp03</t>
-  </si>
-  <si>
-    <t>Escalado agresivo mixto hasta 500 VUs default.</t>
-  </si>
-  <si>
-    <t>Determinar punto de quiebre sistémico y endpoint/componente que falla primero.</t>
-  </si>
-  <si>
-    <t>CP-MIX-06</t>
-  </si>
-  <si>
-    <t>Colapso Sistémico Controlado</t>
-  </si>
-  <si>
-    <t>Mixed Collapse</t>
-  </si>
-  <si>
-    <t>npm run perf:all:collapse</t>
-  </si>
-  <si>
-    <t>Rampa rápida mixta hasta 800 VUs default.</t>
-  </si>
-  <si>
-    <t>Identificar colapso sistémico, errores dominantes y tiempo de recuperación posterior.</t>
   </si>
 </sst>
 </file>
@@ -853,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" style="1" customWidth="1"/>
@@ -1418,180 +1307,6 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="5">
-        <v>19</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>21</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
-        <v>22</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
-        <v>23</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="5">
-        <v>24</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>